<commit_message>
- change paths - softcoding saving section - create new dataframes (due extended lai reference period from 2000)
</commit_message>
<xml_diff>
--- a/output/differences_absolute_local.xlsx
+++ b/output/differences_absolute_local.xlsx
@@ -399,7 +399,7 @@
         <v>0.00860362982925314</v>
       </c>
       <c r="D2">
-        <v>0.1571913580246913</v>
+        <v>0.1846348096348098</v>
       </c>
       <c r="E2" s="2">
         <v>41395</v>
@@ -416,7 +416,7 @@
         <v>-0.02374153000524915</v>
       </c>
       <c r="D3">
-        <v>0.008333333333333304</v>
+        <v>0.1383333333333332</v>
       </c>
       <c r="E3" s="2">
         <v>41426</v>
@@ -433,7 +433,7 @@
         <v>-0.01722897012383309</v>
       </c>
       <c r="D4">
-        <v>0.2513668430335096</v>
+        <v>0.2794949494949495</v>
       </c>
       <c r="E4" s="2">
         <v>41456</v>
@@ -450,7 +450,7 @@
         <v>-0.01406791063742444</v>
       </c>
       <c r="D5">
-        <v>0.06446759259259283</v>
+        <v>0.05068181818181827</v>
       </c>
       <c r="E5" s="2">
         <v>41487</v>
@@ -467,7 +467,7 @@
         <v>-0.01030196646719975</v>
       </c>
       <c r="D6">
-        <v>-0.1088888888888886</v>
+        <v>-0.2111111111111112</v>
       </c>
       <c r="E6" s="2">
         <v>41518</v>
@@ -484,7 +484,7 @@
         <v>-0.01275865997126613</v>
       </c>
       <c r="D7">
-        <v>-0.3261419753086421</v>
+        <v>-0.2986985236985236</v>
       </c>
       <c r="E7" s="2">
         <v>41760</v>
@@ -501,7 +501,7 @@
         <v>-0.03091559301985827</v>
       </c>
       <c r="D8">
-        <v>0.07500000000000018</v>
+        <v>0.2050000000000001</v>
       </c>
       <c r="E8" s="2">
         <v>41791</v>
@@ -518,7 +518,7 @@
         <v>-0.01958511959785458</v>
       </c>
       <c r="D9">
-        <v>-0.1486331569664903</v>
+        <v>-0.1205050505050504</v>
       </c>
       <c r="E9" s="2">
         <v>41821</v>
@@ -535,7 +535,7 @@
         <v>0.00634490228779816</v>
       </c>
       <c r="D10">
-        <v>-0.07442129629629601</v>
+        <v>-0.08820707070707057</v>
       </c>
       <c r="E10" s="2">
         <v>41852</v>
@@ -552,7 +552,7 @@
         <v>0.002243700570631113</v>
       </c>
       <c r="D11">
-        <v>-0.08666666666666645</v>
+        <v>-0.1888888888888891</v>
       </c>
       <c r="E11" s="2">
         <v>41883</v>
@@ -569,7 +569,7 @@
         <v>-0.0137811691051116</v>
       </c>
       <c r="D12">
-        <v>-0.1344753086419748</v>
+        <v>-0.1070318570318562</v>
       </c>
       <c r="E12" s="2">
         <v>42125</v>
@@ -586,7 +586,7 @@
         <v>-0.04540739123045137</v>
       </c>
       <c r="D13">
-        <v>-0.4138888888888892</v>
+        <v>-0.2838888888888893</v>
       </c>
       <c r="E13" s="2">
         <v>42156</v>
@@ -603,7 +603,7 @@
         <v>-0.02874346668081523</v>
       </c>
       <c r="D14">
-        <v>-0.5819664902998238</v>
+        <v>-0.553838383838384</v>
       </c>
       <c r="E14" s="2">
         <v>42186</v>
@@ -620,7 +620,7 @@
         <v>-0.007310047786302148</v>
       </c>
       <c r="D15">
-        <v>0.4033564814814818</v>
+        <v>0.3895707070707073</v>
       </c>
       <c r="E15" s="2">
         <v>42217</v>
@@ -637,7 +637,7 @@
         <v>0.01328954429094964</v>
       </c>
       <c r="D16">
-        <v>0.2577777777777781</v>
+        <v>0.1555555555555554</v>
       </c>
       <c r="E16" s="2">
         <v>42248</v>
@@ -654,7 +654,7 @@
         <v>0.007712613370235405</v>
       </c>
       <c r="D17">
-        <v>0.1905246913580245</v>
+        <v>0.217968142968143</v>
       </c>
       <c r="E17" s="2">
         <v>42491</v>
@@ -671,7 +671,7 @@
         <v>-0.006623607967782663</v>
       </c>
       <c r="D18">
-        <v>0.5416666666666665</v>
+        <v>0.6716666666666664</v>
       </c>
       <c r="E18" s="2">
         <v>42522</v>
@@ -688,7 +688,7 @@
         <v>0.0006351220292883653</v>
       </c>
       <c r="D19">
-        <v>-0.5986331569664904</v>
+        <v>-0.5705050505050506</v>
       </c>
       <c r="E19" s="2">
         <v>42552</v>
@@ -705,7 +705,7 @@
         <v>-0.0310006832078159</v>
       </c>
       <c r="D20">
-        <v>-0.2133101851851853</v>
+        <v>-0.2270959595959599</v>
       </c>
       <c r="E20" s="2">
         <v>42583</v>
@@ -722,7 +722,7 @@
         <v>-0.03512588581019871</v>
       </c>
       <c r="D21">
-        <v>-0.517222222222222</v>
+        <v>-0.6194444444444447</v>
       </c>
       <c r="E21" s="2">
         <v>42614</v>
@@ -739,7 +739,7 @@
         <v>-0.01964168897196528</v>
       </c>
       <c r="D22">
-        <v>-0.03169753086419735</v>
+        <v>-0.004254079254078835</v>
       </c>
       <c r="E22" s="2">
         <v>42856</v>
@@ -756,7 +756,7 @@
         <v>-0.02141427136702215</v>
       </c>
       <c r="D23">
-        <v>-0.4305555555555558</v>
+        <v>-0.3005555555555559</v>
       </c>
       <c r="E23" s="2">
         <v>42887</v>
@@ -773,7 +773,7 @@
         <v>-0.01198174482662986</v>
       </c>
       <c r="D24">
-        <v>-0.3152998236331572</v>
+        <v>-0.2871717171717174</v>
       </c>
       <c r="E24" s="2">
         <v>42917</v>
@@ -790,7 +790,7 @@
         <v>-0.004982195744320211</v>
       </c>
       <c r="D25">
-        <v>-0.04108796296296324</v>
+        <v>-0.0548737373737378</v>
       </c>
       <c r="E25" s="2">
         <v>42948</v>
@@ -807,7 +807,7 @@
         <v>-0.0113364099745534</v>
       </c>
       <c r="D26">
-        <v>-0.7477777777777777</v>
+        <v>-0.8500000000000003</v>
       </c>
       <c r="E26" s="2">
         <v>42979</v>

</xml_diff>